<commit_message>
voice call stall rules and conversation memory
</commit_message>
<xml_diff>
--- a/docs/SwiftLoan-Production-Plan.xlsx
+++ b/docs/SwiftLoan-Production-Plan.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Backend &amp; Infra" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Mobile App'!A1:I47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Mobile App'!A1:I51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2">'Website'!A1:I33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3">'Admin Dashboard'!A1:I39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4">'Backend &amp; Infra'!A1:I49</definedName>
@@ -450,10 +450,10 @@
         <v>Mobile App</v>
       </c>
       <c r="B2">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C2">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D2">
         <v>2</v>
@@ -465,7 +465,7 @@
         <v>22</v>
       </c>
       <c r="G2" t="str">
-        <v>50%</v>
+        <v>54%</v>
       </c>
       <c r="H2">
         <v>11</v>
@@ -554,10 +554,10 @@
         <v>TOTAL</v>
       </c>
       <c r="B7">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C7">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D7">
         <v>7</v>
@@ -569,7 +569,7 @@
         <v>68</v>
       </c>
       <c r="G7" t="str">
-        <v>54%</v>
+        <v>55%</v>
       </c>
       <c r="H7">
         <v>44</v>
@@ -616,7 +616,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I51"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -800,7 +800,7 @@
         <v/>
       </c>
       <c r="I6" t="str">
-        <v>OnePlus Nord AC2001. Needed C:\pg17-style short paths (MAX_PATH)</v>
+        <v>Realme RMX2170 (Android 12). Needed C:\pg17-style short paths (Windows MAX_PATH).</v>
       </c>
     </row>
     <row r="7">
@@ -1568,10 +1568,10 @@
         <v>End-to-end push test to a real handset</v>
       </c>
       <c r="D33" t="str">
-        <v>Not Started</v>
+        <v>Done</v>
       </c>
       <c r="E33" t="str">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="F33" t="str">
         <v>P0</v>
@@ -1580,10 +1580,10 @@
         <v>QA</v>
       </c>
       <c r="H33" t="str">
-        <v>All of the above</v>
+        <v/>
       </c>
       <c r="I33" t="str">
-        <v/>
+        <v>VERIFIED on a real handset: FCM accepted the send (HTTP 200) and the notification rendered in the tray. Sent via FCM HTTP v1 with the service-account key.</v>
       </c>
     </row>
     <row r="34">
@@ -1655,10 +1655,10 @@
         <v>Point in-app agent at api-in.getello.ai (India)</v>
       </c>
       <c r="D36" t="str">
-        <v>Not Started</v>
+        <v>Done</v>
       </c>
       <c r="E36" t="str">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="F36" t="str">
         <v>P1</v>
@@ -1670,7 +1670,7 @@
         <v/>
       </c>
       <c r="I36" t="str">
-        <v>Currently api-dev; server already switched</v>
+        <v>All four clients now on api-in + connect-in with the production key: mobile app, website, admin, server. WebSocket handshake to connect-in verified OPEN.</v>
       </c>
     </row>
     <row r="37">
@@ -1693,13 +1693,13 @@
         <v>P1</v>
       </c>
       <c r="G37" t="str">
-        <v>Ops</v>
+        <v>Dev</v>
       </c>
       <c r="H37" t="str">
         <v/>
       </c>
       <c r="I37" t="str">
-        <v>Prompt lives on the Ello dashboard, not in the repo</v>
+        <v>Prompts now live in prompts/ and are pushed with `npm run ello:sync -- --role companion` — no longer dashboard-only. Still to do: teach the prompt to open from the new userContext brief (MOB-047).</v>
       </c>
     </row>
     <row r="38">
@@ -1992,10 +1992,126 @@
         <v/>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>MOB-047</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Journey tracking</v>
+      </c>
+      <c r="C48" t="str">
+        <v>GET /api/context/me — full history for the signed-in phone, handed to the in-app agent</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Done</v>
+      </c>
+      <c r="E48" t="str">
+        <v>100</v>
+      </c>
+      <c r="F48" t="str">
+        <v>P1</v>
+      </c>
+      <c r="G48" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="H48" t="str">
+        <v/>
+      </c>
+      <c r="I48" t="str">
+        <v>The non-deep-link path: a Play Store install arrives with only a phone number. Returns stage, website enquiries, last call + outcome, application/loan, and a one-line brief the agent can open from. Fetched on login (either route) and passed via registerPageContext.</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>MOB-048</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Upshot SDK</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Fix Upshot native wiring (auth was failing outright)</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Done</v>
+      </c>
+      <c r="E49" t="str">
+        <v>100</v>
+      </c>
+      <c r="F49" t="str">
+        <v>P0</v>
+      </c>
+      <c r="G49" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="H49" t="str">
+        <v/>
+      </c>
+      <c r="I49" t="str">
+        <v>Four hard blockers, not polish: (1) init keys must be bkApplicationID/bkApplicationOwnerID, not AppId/OwnerId — the bridge copies them verbatim, so auth returned "Invalid parameters"; (2) MainApplication must extend UpshotApplication or its static application field stays null; (3) androidx.work missing → NoClassDefFoundError crash on launch; (4) no FirebaseMessagingService existed, so data-only Upshot pushes were silently dropped. Auth now returns status:true.</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>MOB-049</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Notifications</v>
+      </c>
+      <c r="C50" t="str">
+        <v>SMS OTP delivery in production</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Not Started</v>
+      </c>
+      <c r="E50" t="str">
+        <v>0</v>
+      </c>
+      <c r="F50" t="str">
+        <v>P0</v>
+      </c>
+      <c r="G50" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="H50" t="str">
+        <v>SMS provider + DLT registration</v>
+      </c>
+      <c r="I50" t="str">
+        <v>LAUNCH BLOCKER. createOtp() says "in production this is sent via SMS" but NO SMS sender exists (no Twilio/MSG91/Gupshup/Kaleyra/Exotel anywhere). Today the code is returned in the API response for dev/demo and is undefined in production — so nobody can log in to the production app. Needs a DLT-registered Indian sender; template pre-registration takes days (TRAI).</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>MOB-050</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Notifications</v>
+      </c>
+      <c r="C51" t="str">
+        <v>WhatsApp messaging (app link, nudges)</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Not Started</v>
+      </c>
+      <c r="E51" t="str">
+        <v>0</v>
+      </c>
+      <c r="F51" t="str">
+        <v>P1</v>
+      </c>
+      <c r="G51" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="H51" t="str">
+        <v>Upshot WhatsApp channel</v>
+      </c>
+      <c r="I51" t="str">
+        <v>StallRule already accepts whatsapp/sms as channels, but the dispatch queue only handles upshot_event and upshot_user_upsert — nothing sends WhatsApp directly. Delivery is delegated to Upshot campaigns, so it is only as configured as those are. Decide: keep delegating, or add a direct send path alongside MOB-049.</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I47"/>
+  <autoFilter ref="A1:I51"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I47"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I51"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>